<commit_message>
weak anchor placement data added
</commit_message>
<xml_diff>
--- a/data/trilateration_data.xlsx
+++ b/data/trilateration_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emonc\OneDrive\Desktop\RSN Group UWB Project\eece5554-final-project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{93AB14DC-6468-4B1B-98B9-CA2933435031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40F62FD3-9501-4149-9615-251F16AE5E37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{ECF9459F-14D8-4B26-8035-2E30A54B085A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="36">
   <si>
     <t>cm</t>
   </si>
@@ -53,9 +53,6 @@
     <t>id2</t>
   </si>
   <si>
-    <t>calibration data</t>
-  </si>
-  <si>
     <t>anchor locations</t>
   </si>
   <si>
@@ -122,9 +119,6 @@
     <t>id2 (cm)</t>
   </si>
   <si>
-    <t>robot geometry</t>
-  </si>
-  <si>
     <t>corner</t>
   </si>
   <si>
@@ -135,6 +129,24 @@
   </si>
   <si>
     <t>y (in)</t>
+  </si>
+  <si>
+    <t>Weak Anchor Placement Test</t>
+  </si>
+  <si>
+    <t>Ideal Anchor Placement</t>
+  </si>
+  <si>
+    <t>Anchor Locations</t>
+  </si>
+  <si>
+    <t>Robot Geometry</t>
+  </si>
+  <si>
+    <t>Weak Anchor Placement</t>
+  </si>
+  <si>
+    <t>Calibration Data</t>
   </si>
 </sst>
 </file>
@@ -651,7 +663,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
@@ -676,7 +688,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
@@ -697,14 +708,21 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1039,124 +1057,116 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E700C2C4-62D6-4550-AD26-EC19A6843912}">
-  <dimension ref="B1:V30"/>
+  <dimension ref="B1:V42"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
     <col min="2" max="2" width="13.76953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.1328125" customWidth="1"/>
     <col min="4" max="4" width="7.453125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.1796875" style="24" customWidth="1"/>
-    <col min="7" max="7" width="9.1796875" customWidth="1"/>
+    <col min="6" max="7" width="9.1796875" customWidth="1"/>
     <col min="12" max="12" width="11.5" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10.1796875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="11.76953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:22" ht="15.5" thickBot="1" x14ac:dyDescent="0.9"/>
-    <row r="2" spans="2:22" x14ac:dyDescent="0.75">
+    <row r="1" spans="2:17" ht="15.5" thickBot="1" x14ac:dyDescent="0.9"/>
+    <row r="2" spans="2:17" x14ac:dyDescent="0.75">
       <c r="B2" s="20"/>
-      <c r="C2" s="21" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="21"/>
+      <c r="C2" s="45" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="45"/>
       <c r="E2" s="21"/>
       <c r="F2" s="21"/>
       <c r="G2" s="22"/>
       <c r="H2" s="20"/>
-      <c r="I2" s="46" t="s">
-        <v>5</v>
-      </c>
-      <c r="J2" s="46"/>
-      <c r="K2" s="21"/>
+      <c r="I2" s="45" t="s">
+        <v>33</v>
+      </c>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
       <c r="L2" s="22"/>
       <c r="M2" s="20"/>
-      <c r="N2" s="46" t="s">
+      <c r="N2" s="45" t="s">
+        <v>31</v>
+      </c>
+      <c r="O2" s="45"/>
+      <c r="P2" s="45"/>
+      <c r="Q2" s="22"/>
+    </row>
+    <row r="3" spans="2:17" x14ac:dyDescent="0.75">
+      <c r="B3" s="23"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="46" t="s">
         <v>27</v>
       </c>
-      <c r="O2" s="46"/>
-      <c r="P2" s="21"/>
-      <c r="Q2" s="22"/>
-    </row>
-    <row r="3" spans="2:22" x14ac:dyDescent="0.75">
-      <c r="B3" s="23"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="G3" s="25"/>
-      <c r="H3" s="23"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="24"/>
-      <c r="L3" s="25"/>
+      <c r="J3" s="46"/>
+      <c r="K3" s="46"/>
+      <c r="L3" s="24"/>
       <c r="M3" s="23"/>
-      <c r="N3" s="47" t="s">
+      <c r="N3" s="46" t="s">
+        <v>32</v>
+      </c>
+      <c r="O3" s="46"/>
+      <c r="P3" s="46"/>
+      <c r="Q3" s="24"/>
+    </row>
+    <row r="4" spans="2:17" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="B4" s="23"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
+      <c r="E4" s="44"/>
+      <c r="F4" s="44"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="23"/>
+      <c r="L4" s="24"/>
+      <c r="M4" s="23"/>
+      <c r="Q4" s="24"/>
+    </row>
+    <row r="5" spans="2:17" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="B5" s="23"/>
+      <c r="C5" s="41" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="35" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="35" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="36" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="24"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="41" t="s">
+        <v>26</v>
+      </c>
+      <c r="J5" s="35" t="s">
+        <v>28</v>
+      </c>
+      <c r="K5" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="O3" s="47"/>
-      <c r="P3" s="24"/>
-      <c r="Q3" s="25"/>
-    </row>
-    <row r="4" spans="2:22" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="B4" s="23"/>
-      <c r="C4" s="45"/>
-      <c r="D4" s="45"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="45"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="24"/>
-      <c r="J4" s="24"/>
-      <c r="K4" s="24"/>
-      <c r="L4" s="25"/>
-      <c r="M4" s="23"/>
-      <c r="N4" s="24"/>
-      <c r="O4" s="24"/>
-      <c r="P4" s="24"/>
-      <c r="Q4" s="25"/>
-    </row>
-    <row r="5" spans="2:22" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="B5" s="23"/>
-      <c r="C5" s="42" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" s="36" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5" s="36" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" s="37" t="s">
-        <v>26</v>
-      </c>
-      <c r="G5" s="25"/>
-      <c r="H5" s="23"/>
-      <c r="I5" s="45"/>
-      <c r="J5" s="43" t="s">
+      <c r="L5" s="24"/>
+      <c r="M5" s="23"/>
+      <c r="N5" s="44"/>
+      <c r="O5" s="42" t="s">
+        <v>10</v>
+      </c>
+      <c r="P5" s="43" t="s">
         <v>11</v>
       </c>
-      <c r="K5" s="44" t="s">
-        <v>12</v>
-      </c>
-      <c r="L5" s="25"/>
-      <c r="M5" s="23"/>
-      <c r="N5" s="42" t="s">
-        <v>28</v>
-      </c>
-      <c r="O5" s="36" t="s">
-        <v>30</v>
-      </c>
-      <c r="P5" s="37" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q5" s="25"/>
-    </row>
-    <row r="6" spans="2:22" x14ac:dyDescent="0.75">
+      <c r="Q5" s="24"/>
+    </row>
+    <row r="6" spans="2:17" x14ac:dyDescent="0.75">
       <c r="B6" s="23"/>
       <c r="C6" s="18">
         <v>2</v>
       </c>
-      <c r="D6" s="40">
+      <c r="D6" s="39">
         <v>48</v>
       </c>
       <c r="E6" s="4">
@@ -1165,31 +1175,31 @@
       <c r="F6" s="5">
         <v>43</v>
       </c>
-      <c r="G6" s="25"/>
+      <c r="G6" s="24"/>
       <c r="H6" s="23"/>
-      <c r="I6" s="33" t="s">
+      <c r="I6" s="37">
         <v>1</v>
       </c>
-      <c r="J6" s="3">
+      <c r="J6" s="20">
+        <v>20</v>
+      </c>
+      <c r="K6" s="22">
+        <v>-7</v>
+      </c>
+      <c r="L6" s="24"/>
+      <c r="M6" s="23"/>
+      <c r="N6" s="32" t="s">
+        <v>1</v>
+      </c>
+      <c r="O6" s="3">
         <v>0</v>
       </c>
-      <c r="K6" s="29">
+      <c r="P6" s="28">
         <v>0</v>
       </c>
-      <c r="L6" s="25"/>
-      <c r="M6" s="23"/>
-      <c r="N6" s="38">
-        <v>1</v>
-      </c>
-      <c r="O6" s="20">
-        <v>20</v>
-      </c>
-      <c r="P6" s="22">
-        <v>-7</v>
-      </c>
-      <c r="Q6" s="25"/>
-    </row>
-    <row r="7" spans="2:22" x14ac:dyDescent="0.75">
+      <c r="Q6" s="24"/>
+    </row>
+    <row r="7" spans="2:17" x14ac:dyDescent="0.75">
       <c r="B7" s="23"/>
       <c r="C7" s="18">
         <v>4</v>
@@ -1203,31 +1213,31 @@
       <c r="F7" s="7">
         <v>105</v>
       </c>
-      <c r="G7" s="25"/>
+      <c r="G7" s="24"/>
       <c r="H7" s="23"/>
-      <c r="I7" s="34" t="s">
+      <c r="I7" s="37">
         <v>2</v>
       </c>
-      <c r="J7" s="30">
+      <c r="J7" s="23">
+        <v>20</v>
+      </c>
+      <c r="K7" s="24">
+        <v>7</v>
+      </c>
+      <c r="L7" s="24"/>
+      <c r="M7" s="23"/>
+      <c r="N7" s="33" t="s">
+        <v>2</v>
+      </c>
+      <c r="O7" s="29">
         <v>0</v>
       </c>
-      <c r="K7" s="31">
+      <c r="P7" s="30">
         <v>4.5</v>
       </c>
-      <c r="L7" s="25"/>
-      <c r="M7" s="23"/>
-      <c r="N7" s="38">
-        <v>2</v>
-      </c>
-      <c r="O7" s="23">
-        <v>20</v>
-      </c>
-      <c r="P7" s="25">
-        <v>7</v>
-      </c>
-      <c r="Q7" s="25"/>
-    </row>
-    <row r="8" spans="2:22" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="Q7" s="24"/>
+    </row>
+    <row r="8" spans="2:17" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
       <c r="B8" s="23"/>
       <c r="C8" s="18">
         <v>6</v>
@@ -1241,31 +1251,31 @@
       <c r="F8" s="7">
         <v>177</v>
       </c>
-      <c r="G8" s="25"/>
+      <c r="G8" s="24"/>
       <c r="H8" s="23"/>
-      <c r="I8" s="35" t="s">
+      <c r="I8" s="37">
         <v>3</v>
       </c>
-      <c r="J8" s="32">
+      <c r="J8" s="23">
+        <v>0</v>
+      </c>
+      <c r="K8" s="24">
+        <v>7</v>
+      </c>
+      <c r="L8" s="24"/>
+      <c r="M8" s="23"/>
+      <c r="N8" s="34" t="s">
+        <v>3</v>
+      </c>
+      <c r="O8" s="31">
         <v>4.5</v>
       </c>
-      <c r="K8" s="10">
+      <c r="P8" s="10">
         <v>0</v>
       </c>
-      <c r="L8" s="25"/>
-      <c r="M8" s="23"/>
-      <c r="N8" s="38">
-        <v>3</v>
-      </c>
-      <c r="O8" s="23">
-        <v>0</v>
-      </c>
-      <c r="P8" s="25">
-        <v>7</v>
-      </c>
-      <c r="Q8" s="25"/>
-    </row>
-    <row r="9" spans="2:22" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="Q8" s="24"/>
+    </row>
+    <row r="9" spans="2:17" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
       <c r="B9" s="23"/>
       <c r="C9" s="18">
         <v>8</v>
@@ -1279,25 +1289,22 @@
       <c r="F9" s="7">
         <v>225</v>
       </c>
-      <c r="G9" s="25"/>
+      <c r="G9" s="24"/>
       <c r="H9" s="23"/>
-      <c r="I9" s="24"/>
-      <c r="J9" s="24"/>
-      <c r="K9" s="24"/>
-      <c r="L9" s="25"/>
+      <c r="I9" s="38">
+        <v>4</v>
+      </c>
+      <c r="J9" s="25">
+        <v>0</v>
+      </c>
+      <c r="K9" s="27">
+        <v>-7</v>
+      </c>
+      <c r="L9" s="24"/>
       <c r="M9" s="23"/>
-      <c r="N9" s="39">
-        <v>4</v>
-      </c>
-      <c r="O9" s="26">
-        <v>0</v>
-      </c>
-      <c r="P9" s="28">
-        <v>-7</v>
-      </c>
-      <c r="Q9" s="25"/>
-    </row>
-    <row r="10" spans="2:22" x14ac:dyDescent="0.75">
+      <c r="Q9" s="24"/>
+    </row>
+    <row r="10" spans="2:17" x14ac:dyDescent="0.75">
       <c r="B10" s="23"/>
       <c r="C10" s="18">
         <v>10</v>
@@ -1311,19 +1318,13 @@
       <c r="F10" s="7">
         <v>306</v>
       </c>
-      <c r="G10" s="25"/>
+      <c r="G10" s="24"/>
       <c r="H10" s="23"/>
-      <c r="I10" s="24"/>
-      <c r="J10" s="24"/>
-      <c r="K10" s="24"/>
-      <c r="L10" s="25"/>
+      <c r="L10" s="24"/>
       <c r="M10" s="23"/>
-      <c r="N10" s="24"/>
-      <c r="O10" s="24"/>
-      <c r="P10" s="24"/>
-      <c r="Q10" s="25"/>
-    </row>
-    <row r="11" spans="2:22" x14ac:dyDescent="0.75">
+      <c r="Q10" s="24"/>
+    </row>
+    <row r="11" spans="2:17" x14ac:dyDescent="0.75">
       <c r="B11" s="23"/>
       <c r="C11" s="18">
         <v>12</v>
@@ -1337,19 +1338,13 @@
       <c r="F11" s="7">
         <v>393</v>
       </c>
-      <c r="G11" s="25"/>
+      <c r="G11" s="24"/>
       <c r="H11" s="23"/>
-      <c r="I11" s="24"/>
-      <c r="J11" s="24"/>
-      <c r="K11" s="24"/>
-      <c r="L11" s="25"/>
+      <c r="L11" s="24"/>
       <c r="M11" s="23"/>
-      <c r="N11" s="24"/>
-      <c r="O11" s="24"/>
-      <c r="P11" s="24"/>
-      <c r="Q11" s="25"/>
-    </row>
-    <row r="12" spans="2:22" x14ac:dyDescent="0.75">
+      <c r="Q11" s="24"/>
+    </row>
+    <row r="12" spans="2:17" x14ac:dyDescent="0.75">
       <c r="B12" s="23"/>
       <c r="C12" s="18">
         <v>14</v>
@@ -1363,19 +1358,13 @@
       <c r="F12" s="7">
         <v>424</v>
       </c>
-      <c r="G12" s="25"/>
+      <c r="G12" s="24"/>
       <c r="H12" s="23"/>
-      <c r="I12" s="24"/>
-      <c r="J12" s="24"/>
-      <c r="K12" s="24"/>
-      <c r="L12" s="25"/>
+      <c r="L12" s="24"/>
       <c r="M12" s="23"/>
-      <c r="N12" s="24"/>
-      <c r="O12" s="24"/>
-      <c r="P12" s="24"/>
-      <c r="Q12" s="25"/>
-    </row>
-    <row r="13" spans="2:22" x14ac:dyDescent="0.75">
+      <c r="Q12" s="24"/>
+    </row>
+    <row r="13" spans="2:17" x14ac:dyDescent="0.75">
       <c r="B13" s="23"/>
       <c r="C13" s="18">
         <v>16</v>
@@ -1389,19 +1378,13 @@
       <c r="F13" s="7">
         <v>491</v>
       </c>
-      <c r="G13" s="25"/>
+      <c r="G13" s="24"/>
       <c r="H13" s="23"/>
-      <c r="I13" s="24"/>
-      <c r="J13" s="24"/>
-      <c r="K13" s="24"/>
-      <c r="L13" s="25"/>
+      <c r="L13" s="24"/>
       <c r="M13" s="23"/>
-      <c r="N13" s="24"/>
-      <c r="O13" s="24"/>
-      <c r="P13" s="24"/>
-      <c r="Q13" s="25"/>
-    </row>
-    <row r="14" spans="2:22" x14ac:dyDescent="0.75">
+      <c r="Q13" s="24"/>
+    </row>
+    <row r="14" spans="2:17" x14ac:dyDescent="0.75">
       <c r="B14" s="23"/>
       <c r="C14" s="18">
         <v>18</v>
@@ -1415,24 +1398,18 @@
       <c r="F14" s="7">
         <v>590</v>
       </c>
-      <c r="G14" s="25"/>
+      <c r="G14" s="24"/>
       <c r="H14" s="23"/>
-      <c r="I14" s="24"/>
-      <c r="J14" s="24"/>
-      <c r="K14" s="24"/>
-      <c r="L14" s="25"/>
+      <c r="L14" s="24"/>
       <c r="M14" s="23"/>
-      <c r="N14" s="24"/>
-      <c r="O14" s="24"/>
-      <c r="P14" s="24"/>
-      <c r="Q14" s="25"/>
-    </row>
-    <row r="15" spans="2:22" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="Q14" s="24"/>
+    </row>
+    <row r="15" spans="2:17" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
       <c r="B15" s="23"/>
       <c r="C15" s="19">
         <v>20</v>
       </c>
-      <c r="D15" s="41">
+      <c r="D15" s="40">
         <v>650</v>
       </c>
       <c r="E15" s="9">
@@ -1441,65 +1418,47 @@
       <c r="F15" s="10">
         <v>611</v>
       </c>
-      <c r="G15" s="25"/>
+      <c r="G15" s="24"/>
       <c r="H15" s="23"/>
-      <c r="I15" s="24"/>
-      <c r="J15" s="24"/>
-      <c r="K15" s="24"/>
-      <c r="L15" s="25"/>
+      <c r="L15" s="24"/>
       <c r="M15" s="23"/>
-      <c r="N15" s="24"/>
-      <c r="O15" s="24"/>
-      <c r="P15" s="24"/>
-      <c r="Q15" s="25"/>
-    </row>
-    <row r="16" spans="2:22" s="24" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="Q15" s="24"/>
+    </row>
+    <row r="16" spans="2:17" x14ac:dyDescent="0.75">
       <c r="B16" s="23"/>
-      <c r="G16" s="25"/>
+      <c r="G16" s="24"/>
       <c r="H16" s="23"/>
-      <c r="L16" s="25"/>
+      <c r="L16" s="24"/>
       <c r="M16" s="23"/>
-      <c r="Q16" s="25"/>
-      <c r="R16"/>
-      <c r="S16"/>
-      <c r="T16"/>
-      <c r="U16"/>
-      <c r="V16"/>
+      <c r="Q16" s="24"/>
     </row>
     <row r="17" spans="2:22" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="B17" s="26"/>
-      <c r="C17" s="27"/>
-      <c r="D17" s="27"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="28"/>
+      <c r="B17" s="25"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="27"/>
       <c r="H17" s="23"/>
-      <c r="I17" s="24"/>
-      <c r="J17" s="24"/>
-      <c r="K17" s="24"/>
-      <c r="L17" s="25"/>
+      <c r="L17" s="24"/>
       <c r="M17" s="23"/>
-      <c r="N17" s="24"/>
-      <c r="O17" s="24"/>
-      <c r="P17" s="24"/>
-      <c r="Q17" s="25"/>
-      <c r="R17" s="24"/>
-      <c r="S17" s="24"/>
-      <c r="T17" s="24"/>
-      <c r="U17" s="24"/>
-      <c r="V17" s="24"/>
+      <c r="Q17" s="24"/>
     </row>
     <row r="18" spans="2:22" x14ac:dyDescent="0.75">
       <c r="B18" s="20"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
+      <c r="C18" s="45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" s="45"/>
+      <c r="E18" s="45"/>
       <c r="F18" s="21"/>
       <c r="G18" s="22"/>
       <c r="H18" s="20"/>
-      <c r="I18" s="21"/>
-      <c r="J18" s="21"/>
-      <c r="K18" s="21"/>
+      <c r="I18" s="45" t="s">
+        <v>31</v>
+      </c>
+      <c r="J18" s="45"/>
+      <c r="K18" s="45"/>
       <c r="L18" s="21"/>
       <c r="M18" s="21"/>
       <c r="N18" s="21"/>
@@ -1514,114 +1473,86 @@
     </row>
     <row r="19" spans="2:22" x14ac:dyDescent="0.75">
       <c r="B19" s="23"/>
-      <c r="C19" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="G19" s="25"/>
+      <c r="C19" s="46" t="s">
+        <v>21</v>
+      </c>
+      <c r="D19" s="46"/>
+      <c r="E19" s="46"/>
+      <c r="G19" s="24"/>
       <c r="H19" s="23"/>
-      <c r="I19" s="24" t="s">
-        <v>21</v>
-      </c>
-      <c r="J19" s="24"/>
-      <c r="K19" s="24"/>
-      <c r="L19" s="24"/>
-      <c r="M19" s="24"/>
-      <c r="N19" s="24"/>
-      <c r="O19" s="24"/>
-      <c r="P19" s="24"/>
-      <c r="Q19" s="24"/>
-      <c r="R19" s="24"/>
-      <c r="S19" s="24"/>
-      <c r="T19" s="24"/>
-      <c r="U19" s="24"/>
-      <c r="V19" s="25"/>
+      <c r="I19" s="46" t="s">
+        <v>20</v>
+      </c>
+      <c r="J19" s="46"/>
+      <c r="K19" s="46"/>
+      <c r="V19" s="24"/>
     </row>
     <row r="20" spans="2:22" x14ac:dyDescent="0.75">
       <c r="B20" s="23"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
-      <c r="G20" s="25"/>
+      <c r="G20" s="24"/>
       <c r="H20" s="23"/>
-      <c r="I20" s="24"/>
-      <c r="J20" s="24"/>
-      <c r="K20" s="24"/>
-      <c r="L20" s="24"/>
-      <c r="M20" s="24"/>
-      <c r="N20" s="24"/>
-      <c r="O20" s="24"/>
-      <c r="P20" s="24"/>
-      <c r="Q20" s="24"/>
-      <c r="R20" s="24"/>
-      <c r="S20" s="24"/>
-      <c r="T20" s="24"/>
-      <c r="U20" s="24"/>
-      <c r="V20" s="25"/>
+      <c r="V20" s="24"/>
     </row>
     <row r="21" spans="2:22" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
       <c r="B21" s="23"/>
-      <c r="C21" s="45" t="s">
-        <v>15</v>
-      </c>
-      <c r="D21" s="45" t="s">
-        <v>10</v>
-      </c>
-      <c r="E21" s="45"/>
-      <c r="F21" s="45" t="s">
+      <c r="C21" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="G21" s="25"/>
+      <c r="D21" s="44" t="s">
+        <v>9</v>
+      </c>
+      <c r="E21" s="44"/>
+      <c r="F21" s="44" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="24"/>
       <c r="H21" s="23"/>
-      <c r="I21" s="45" t="s">
-        <v>15</v>
-      </c>
-      <c r="J21" s="45" t="s">
+      <c r="I21" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="J21" s="44" t="s">
+        <v>5</v>
+      </c>
+      <c r="K21" s="44" t="s">
+        <v>0</v>
+      </c>
+      <c r="L21" s="44"/>
+      <c r="M21" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="K21" s="45" t="s">
+      <c r="N21" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="L21" s="45"/>
-      <c r="M21" s="48" t="s">
+      <c r="O21" s="44"/>
+      <c r="P21" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="N21" s="48" t="s">
+      <c r="Q21" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="O21" s="48"/>
-      <c r="P21" s="45" t="s">
+      <c r="R21" s="44"/>
+      <c r="S21" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="Q21" s="45" t="s">
+      <c r="T21" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="R21" s="45"/>
-      <c r="S21" s="45" t="s">
-        <v>9</v>
-      </c>
-      <c r="T21" s="45" t="s">
-        <v>0</v>
-      </c>
-      <c r="U21" s="45"/>
-      <c r="V21" s="25"/>
+      <c r="U21" s="44"/>
+      <c r="V21" s="24"/>
     </row>
     <row r="22" spans="2:22" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
       <c r="B22" s="23"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="45" t="s">
+      <c r="D22" s="44" t="s">
+        <v>10</v>
+      </c>
+      <c r="E22" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="E22" s="45" t="s">
+      <c r="F22" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="F22" s="45" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" s="25"/>
+      <c r="G22" s="24"/>
       <c r="H22" s="23"/>
-      <c r="I22" s="24"/>
       <c r="J22" s="14" t="s">
         <v>1</v>
       </c>
@@ -1658,12 +1589,12 @@
       <c r="U22" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="V22" s="25"/>
+      <c r="V22" s="24"/>
     </row>
     <row r="23" spans="2:22" x14ac:dyDescent="0.75">
       <c r="B23" s="23"/>
       <c r="C23" s="17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D23" s="20">
         <v>6</v>
@@ -1674,10 +1605,10 @@
       <c r="F23" s="22">
         <v>0</v>
       </c>
-      <c r="G23" s="25"/>
+      <c r="G23" s="24"/>
       <c r="H23" s="23"/>
       <c r="I23" s="17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J23" s="11">
         <v>217</v>
@@ -1715,27 +1646,27 @@
       <c r="U23" s="13">
         <v>183</v>
       </c>
-      <c r="V23" s="25"/>
+      <c r="V23" s="24"/>
     </row>
     <row r="24" spans="2:22" x14ac:dyDescent="0.75">
       <c r="B24" s="23"/>
       <c r="C24" s="18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D24" s="23">
         <v>13.5</v>
       </c>
-      <c r="E24" s="24">
+      <c r="E24">
         <v>7</v>
       </c>
-      <c r="F24" s="25">
+      <c r="F24" s="24">
         <f>180-34.85</f>
         <v>145.15</v>
       </c>
-      <c r="G24" s="25"/>
+      <c r="G24" s="24"/>
       <c r="H24" s="23"/>
       <c r="I24" s="18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J24" s="6">
         <v>523</v>
@@ -1773,27 +1704,27 @@
       <c r="U24" s="7">
         <v>356</v>
       </c>
-      <c r="V24" s="25"/>
+      <c r="V24" s="24"/>
     </row>
     <row r="25" spans="2:22" x14ac:dyDescent="0.75">
       <c r="B25" s="23"/>
       <c r="C25" s="18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D25" s="23">
         <v>18.5</v>
       </c>
-      <c r="E25" s="24">
+      <c r="E25">
         <v>6</v>
       </c>
-      <c r="F25" s="25">
+      <c r="F25" s="24">
         <f>270+ 16.6</f>
         <v>286.60000000000002</v>
       </c>
-      <c r="G25" s="25"/>
+      <c r="G25" s="24"/>
       <c r="H25" s="23"/>
       <c r="I25" s="18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J25" s="6">
         <v>567</v>
@@ -1831,26 +1762,26 @@
       <c r="U25" s="7">
         <v>461</v>
       </c>
-      <c r="V25" s="25"/>
+      <c r="V25" s="24"/>
     </row>
     <row r="26" spans="2:22" x14ac:dyDescent="0.75">
       <c r="B26" s="23"/>
       <c r="C26" s="18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D26" s="23">
         <v>23.5</v>
       </c>
-      <c r="E26" s="24">
+      <c r="E26">
         <v>10</v>
       </c>
-      <c r="F26" s="25">
+      <c r="F26" s="24">
         <v>270</v>
       </c>
-      <c r="G26" s="25"/>
+      <c r="G26" s="24"/>
       <c r="H26" s="23"/>
       <c r="I26" s="18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J26" s="6">
         <v>753</v>
@@ -1888,26 +1819,26 @@
       <c r="U26" s="7">
         <v>648</v>
       </c>
-      <c r="V26" s="25"/>
+      <c r="V26" s="24"/>
     </row>
     <row r="27" spans="2:22" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
       <c r="B27" s="23"/>
       <c r="C27" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="D27" s="26">
+        <v>19</v>
+      </c>
+      <c r="D27" s="25">
         <v>12</v>
       </c>
-      <c r="E27" s="27">
+      <c r="E27" s="26">
         <v>1</v>
       </c>
-      <c r="F27" s="28">
+      <c r="F27" s="27">
         <v>180</v>
       </c>
-      <c r="G27" s="25"/>
+      <c r="G27" s="24"/>
       <c r="H27" s="23"/>
       <c r="I27" s="19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J27" s="8">
         <v>423</v>
@@ -1945,80 +1876,428 @@
       <c r="U27" s="10">
         <v>213</v>
       </c>
-      <c r="V27" s="25"/>
+      <c r="V27" s="24"/>
     </row>
     <row r="28" spans="2:22" x14ac:dyDescent="0.75">
       <c r="B28" s="23"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="G28" s="25"/>
+      <c r="G28" s="24"/>
       <c r="H28" s="23"/>
-      <c r="I28" s="24"/>
-      <c r="J28" s="24"/>
-      <c r="K28" s="24"/>
-      <c r="L28" s="24"/>
-      <c r="M28" s="24"/>
-      <c r="N28" s="24"/>
-      <c r="O28" s="24"/>
-      <c r="P28" s="24"/>
-      <c r="Q28" s="24"/>
-      <c r="R28" s="24"/>
-      <c r="S28" s="24"/>
-      <c r="T28" s="24"/>
-      <c r="U28" s="24"/>
-      <c r="V28" s="25"/>
+      <c r="V28" s="24"/>
     </row>
     <row r="29" spans="2:22" x14ac:dyDescent="0.75">
       <c r="B29" s="23"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
-      <c r="G29" s="25"/>
+      <c r="G29" s="24"/>
       <c r="H29" s="23"/>
-      <c r="I29" s="24"/>
-      <c r="J29" s="24"/>
-      <c r="K29" s="24"/>
-      <c r="L29" s="24"/>
-      <c r="M29" s="24"/>
-      <c r="N29" s="24"/>
-      <c r="O29" s="24"/>
-      <c r="P29" s="24"/>
-      <c r="Q29" s="24"/>
-      <c r="R29" s="24"/>
-      <c r="S29" s="24"/>
-      <c r="T29" s="24"/>
-      <c r="U29" s="24"/>
-      <c r="V29" s="25"/>
+      <c r="V29" s="24"/>
     </row>
     <row r="30" spans="2:22" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
-      <c r="B30" s="26"/>
-      <c r="C30" s="27"/>
-      <c r="D30" s="27"/>
-      <c r="E30" s="27"/>
-      <c r="F30" s="27"/>
-      <c r="G30" s="28"/>
-      <c r="H30" s="26"/>
-      <c r="I30" s="27"/>
-      <c r="J30" s="27"/>
-      <c r="K30" s="27"/>
-      <c r="L30" s="27"/>
-      <c r="M30" s="27"/>
-      <c r="N30" s="27"/>
-      <c r="O30" s="27"/>
-      <c r="P30" s="27"/>
-      <c r="Q30" s="27"/>
-      <c r="R30" s="27"/>
-      <c r="S30" s="27"/>
-      <c r="T30" s="27"/>
-      <c r="U30" s="27"/>
-      <c r="V30" s="28"/>
+      <c r="B30" s="25"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="26"/>
+      <c r="G30" s="27"/>
+      <c r="H30" s="25"/>
+      <c r="I30" s="26"/>
+      <c r="J30" s="26"/>
+      <c r="K30" s="26"/>
+      <c r="L30" s="26"/>
+      <c r="M30" s="26"/>
+      <c r="N30" s="26"/>
+      <c r="O30" s="26"/>
+      <c r="P30" s="26"/>
+      <c r="Q30" s="26"/>
+      <c r="R30" s="26"/>
+      <c r="S30" s="26"/>
+      <c r="T30" s="26"/>
+      <c r="U30" s="26"/>
+      <c r="V30" s="27"/>
+    </row>
+    <row r="31" spans="2:22" x14ac:dyDescent="0.75">
+      <c r="B31" s="20"/>
+      <c r="C31" s="21"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="21"/>
+      <c r="G31" s="22"/>
+      <c r="H31" s="20"/>
+      <c r="I31" s="21"/>
+      <c r="J31" s="21"/>
+      <c r="K31" s="21"/>
+      <c r="L31" s="21"/>
+      <c r="M31" s="21"/>
+      <c r="N31" s="21"/>
+      <c r="O31" s="21"/>
+      <c r="P31" s="21"/>
+      <c r="Q31" s="21"/>
+      <c r="R31" s="21"/>
+      <c r="S31" s="21"/>
+      <c r="T31" s="21"/>
+      <c r="U31" s="21"/>
+      <c r="V31" s="22"/>
+    </row>
+    <row r="32" spans="2:22" x14ac:dyDescent="0.75">
+      <c r="B32" s="23"/>
+      <c r="C32" s="48" t="s">
+        <v>30</v>
+      </c>
+      <c r="D32" s="48"/>
+      <c r="E32" s="48"/>
+      <c r="F32" s="47"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="23"/>
+      <c r="I32" s="47" t="s">
+        <v>34</v>
+      </c>
+      <c r="J32" s="47"/>
+      <c r="K32" s="47"/>
+      <c r="L32" s="47"/>
+      <c r="M32" s="47"/>
+      <c r="N32" s="47"/>
+      <c r="O32" s="47"/>
+      <c r="P32" s="47"/>
+      <c r="Q32" s="47"/>
+      <c r="R32" s="47"/>
+      <c r="S32" s="47"/>
+      <c r="T32" s="47"/>
+      <c r="U32" s="47"/>
+      <c r="V32" s="24"/>
+    </row>
+    <row r="33" spans="2:22" x14ac:dyDescent="0.75">
+      <c r="B33" s="23"/>
+      <c r="C33" s="48" t="s">
+        <v>4</v>
+      </c>
+      <c r="D33" s="48"/>
+      <c r="E33" s="48"/>
+      <c r="F33" s="47"/>
+      <c r="G33" s="24"/>
+      <c r="H33" s="23"/>
+      <c r="I33" s="47"/>
+      <c r="J33" s="47"/>
+      <c r="K33" s="47"/>
+      <c r="L33" s="47"/>
+      <c r="M33" s="47"/>
+      <c r="N33" s="47"/>
+      <c r="O33" s="47"/>
+      <c r="P33" s="47"/>
+      <c r="Q33" s="47"/>
+      <c r="R33" s="47"/>
+      <c r="S33" s="47"/>
+      <c r="T33" s="47"/>
+      <c r="U33" s="47"/>
+      <c r="V33" s="24"/>
+    </row>
+    <row r="34" spans="2:22" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="B34" s="23"/>
+      <c r="C34" s="47"/>
+      <c r="D34" s="47"/>
+      <c r="E34" s="47"/>
+      <c r="F34" s="47"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="23"/>
+      <c r="I34" s="49" t="s">
+        <v>14</v>
+      </c>
+      <c r="J34" s="49" t="s">
+        <v>5</v>
+      </c>
+      <c r="K34" s="49" t="s">
+        <v>0</v>
+      </c>
+      <c r="L34" s="49"/>
+      <c r="M34" s="49" t="s">
+        <v>6</v>
+      </c>
+      <c r="N34" s="49" t="s">
+        <v>0</v>
+      </c>
+      <c r="O34" s="49"/>
+      <c r="P34" s="49" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q34" s="49" t="s">
+        <v>0</v>
+      </c>
+      <c r="R34" s="49"/>
+      <c r="S34" s="49" t="s">
+        <v>8</v>
+      </c>
+      <c r="T34" s="49" t="s">
+        <v>0</v>
+      </c>
+      <c r="U34" s="49"/>
+      <c r="V34" s="24"/>
+    </row>
+    <row r="35" spans="2:22" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="B35" s="23"/>
+      <c r="C35" s="49"/>
+      <c r="D35" s="42" t="s">
+        <v>10</v>
+      </c>
+      <c r="E35" s="43" t="s">
+        <v>11</v>
+      </c>
+      <c r="F35" s="47"/>
+      <c r="G35" s="24"/>
+      <c r="H35" s="23"/>
+      <c r="I35" s="47"/>
+      <c r="J35" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="K35" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="L35" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="M35" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="N35" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="O35" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="P35" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q35" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="R35" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="S35" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="T35" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="U35" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="V35" s="24"/>
+    </row>
+    <row r="36" spans="2:22" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="B36" s="23"/>
+      <c r="C36" s="32" t="s">
+        <v>1</v>
+      </c>
+      <c r="D36" s="3">
+        <v>0</v>
+      </c>
+      <c r="E36" s="28">
+        <v>0</v>
+      </c>
+      <c r="F36" s="47"/>
+      <c r="G36" s="24"/>
+      <c r="H36" s="23"/>
+      <c r="I36" s="41" t="s">
+        <v>15</v>
+      </c>
+      <c r="J36" s="50">
+        <v>209</v>
+      </c>
+      <c r="K36" s="51">
+        <v>189</v>
+      </c>
+      <c r="L36" s="52">
+        <v>211</v>
+      </c>
+      <c r="M36" s="50">
+        <v>166</v>
+      </c>
+      <c r="N36" s="51">
+        <v>134</v>
+      </c>
+      <c r="O36" s="52">
+        <v>153</v>
+      </c>
+      <c r="P36" s="50">
+        <v>204</v>
+      </c>
+      <c r="Q36" s="51">
+        <v>173</v>
+      </c>
+      <c r="R36" s="52">
+        <v>194</v>
+      </c>
+      <c r="S36" s="50">
+        <v>236</v>
+      </c>
+      <c r="T36" s="51">
+        <v>181</v>
+      </c>
+      <c r="U36" s="52">
+        <v>187</v>
+      </c>
+      <c r="V36" s="24"/>
+    </row>
+    <row r="37" spans="2:22" x14ac:dyDescent="0.75">
+      <c r="B37" s="23"/>
+      <c r="C37" s="33" t="s">
+        <v>2</v>
+      </c>
+      <c r="D37" s="29">
+        <v>0</v>
+      </c>
+      <c r="E37" s="30">
+        <v>1</v>
+      </c>
+      <c r="F37" s="47"/>
+      <c r="G37" s="24"/>
+      <c r="H37" s="23"/>
+      <c r="I37" s="47"/>
+      <c r="J37" s="47"/>
+      <c r="K37" s="47"/>
+      <c r="L37" s="47"/>
+      <c r="M37" s="47"/>
+      <c r="N37" s="47"/>
+      <c r="O37" s="47"/>
+      <c r="P37" s="47"/>
+      <c r="Q37" s="47"/>
+      <c r="R37" s="47"/>
+      <c r="S37" s="47"/>
+      <c r="T37" s="47"/>
+      <c r="U37" s="47"/>
+      <c r="V37" s="24"/>
+    </row>
+    <row r="38" spans="2:22" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="B38" s="23"/>
+      <c r="C38" s="34" t="s">
+        <v>3</v>
+      </c>
+      <c r="D38" s="31">
+        <v>1</v>
+      </c>
+      <c r="E38" s="10">
+        <v>0</v>
+      </c>
+      <c r="F38" s="47"/>
+      <c r="G38" s="24"/>
+      <c r="H38" s="23"/>
+      <c r="I38" s="47"/>
+      <c r="J38" s="47"/>
+      <c r="K38" s="47"/>
+      <c r="L38" s="47"/>
+      <c r="M38" s="47"/>
+      <c r="N38" s="47"/>
+      <c r="O38" s="47"/>
+      <c r="P38" s="47"/>
+      <c r="Q38" s="47"/>
+      <c r="R38" s="47"/>
+      <c r="S38" s="47"/>
+      <c r="T38" s="47"/>
+      <c r="U38" s="47"/>
+      <c r="V38" s="24"/>
+    </row>
+    <row r="39" spans="2:22" x14ac:dyDescent="0.75">
+      <c r="B39" s="23"/>
+      <c r="C39" s="47"/>
+      <c r="D39" s="47"/>
+      <c r="E39" s="47"/>
+      <c r="F39" s="47"/>
+      <c r="G39" s="24"/>
+      <c r="H39" s="23"/>
+      <c r="I39" s="47"/>
+      <c r="J39" s="47"/>
+      <c r="K39" s="47"/>
+      <c r="L39" s="47"/>
+      <c r="M39" s="47"/>
+      <c r="N39" s="47"/>
+      <c r="O39" s="47"/>
+      <c r="P39" s="47"/>
+      <c r="Q39" s="47"/>
+      <c r="R39" s="47"/>
+      <c r="S39" s="47"/>
+      <c r="T39" s="47"/>
+      <c r="U39" s="47"/>
+      <c r="V39" s="24"/>
+    </row>
+    <row r="40" spans="2:22" x14ac:dyDescent="0.75">
+      <c r="B40" s="23"/>
+      <c r="C40" s="47"/>
+      <c r="D40" s="47"/>
+      <c r="E40" s="47"/>
+      <c r="F40" s="47"/>
+      <c r="G40" s="24"/>
+      <c r="H40" s="23"/>
+      <c r="I40" s="47"/>
+      <c r="J40" s="47"/>
+      <c r="K40" s="47"/>
+      <c r="L40" s="47"/>
+      <c r="M40" s="47"/>
+      <c r="N40" s="47"/>
+      <c r="O40" s="47"/>
+      <c r="P40" s="47"/>
+      <c r="Q40" s="47"/>
+      <c r="R40" s="47"/>
+      <c r="S40" s="47"/>
+      <c r="T40" s="47"/>
+      <c r="U40" s="47"/>
+      <c r="V40" s="24"/>
+    </row>
+    <row r="41" spans="2:22" x14ac:dyDescent="0.75">
+      <c r="B41" s="23"/>
+      <c r="C41" s="47"/>
+      <c r="D41" s="47"/>
+      <c r="E41" s="47"/>
+      <c r="F41" s="47"/>
+      <c r="G41" s="24"/>
+      <c r="H41" s="23"/>
+      <c r="I41" s="47"/>
+      <c r="J41" s="47"/>
+      <c r="K41" s="47"/>
+      <c r="L41" s="47"/>
+      <c r="M41" s="47"/>
+      <c r="N41" s="47"/>
+      <c r="O41" s="47"/>
+      <c r="P41" s="47"/>
+      <c r="Q41" s="47"/>
+      <c r="R41" s="47"/>
+      <c r="S41" s="47"/>
+      <c r="T41" s="47"/>
+      <c r="U41" s="47"/>
+      <c r="V41" s="24"/>
+    </row>
+    <row r="42" spans="2:22" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
+      <c r="B42" s="25"/>
+      <c r="C42" s="26"/>
+      <c r="D42" s="26"/>
+      <c r="E42" s="26"/>
+      <c r="F42" s="26"/>
+      <c r="G42" s="27"/>
+      <c r="H42" s="25"/>
+      <c r="I42" s="26"/>
+      <c r="J42" s="26"/>
+      <c r="K42" s="26"/>
+      <c r="L42" s="26"/>
+      <c r="M42" s="26"/>
+      <c r="N42" s="26"/>
+      <c r="O42" s="26"/>
+      <c r="P42" s="26"/>
+      <c r="Q42" s="26"/>
+      <c r="R42" s="26"/>
+      <c r="S42" s="26"/>
+      <c r="T42" s="26"/>
+      <c r="U42" s="26"/>
+      <c r="V42" s="27"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="N2:O2"/>
-    <mergeCell ref="N3:O3"/>
+  <mergeCells count="11">
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="I18:K18"/>
+    <mergeCell ref="I19:K19"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="N2:P2"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="I3:K3"/>
+    <mergeCell ref="I2:K2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>